<commit_message>
Add map-ready 'Military Burden Map' sheet to SIPRI workbook
New sheet lists all 172 countries with military burden (% of GDP), ISO3
code, and SIPRI legend band, with each band cell shaded to the SIPRI
colour scheme and a legend/notes block. The Country + Burden columns feed
Excel's Insert > Maps > Filled Map to reproduce the choropleth natively.

make_map_excel.py regenerates the sheet from the workbook's top-40 figures
plus the SIPRI database values, so it stays in sync with the HTML map.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xaim2Fr7Zv9VVTJ6KQGu17
</commit_message>
<xml_diff>
--- a/SIPRI_Military_Expenditure_2025.xlsx
+++ b/SIPRI_Military_Expenditure_2025.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Top 40 Spenders 2025" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Regions &amp; Subregions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="World Share (Top 15)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="World Totals &amp; Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Military Burden Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Regions &amp; Subregions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="World Share (Top 15)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="World Totals &amp; Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +39,38 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1C3F5F"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF5B6672"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="FF1B2430"/>
+    </font>
+    <font>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF5B6672"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -54,8 +87,53 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1C3F5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5D5D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC4D8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F74A3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDC9A34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFECD992"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6D93BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF93B4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5EFD8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -77,11 +155,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCED4DA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCED4DA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCED4DA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCED4DA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,6 +182,60 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -552,7 +698,6 @@
       <c r="I2" t="n">
         <v>33</v>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -656,7 +801,6 @@
       <c r="I5" t="n">
         <v>3.9</v>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -688,7 +832,6 @@
       <c r="I6" t="n">
         <v>3.2</v>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -740,7 +883,6 @@
       <c r="I8" t="n">
         <v>3.1</v>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -844,7 +986,6 @@
       <c r="I11" t="n">
         <v>2.4</v>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -876,7 +1017,6 @@
       <c r="I12" t="n">
         <v>2.2</v>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -928,7 +1068,6 @@
       <c r="I14" t="n">
         <v>1.7</v>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -960,7 +1099,6 @@
       <c r="I15" t="n">
         <v>1.7</v>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -992,7 +1130,6 @@
       <c r="I16" t="n">
         <v>1.7</v>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1024,7 +1161,6 @@
       <c r="I17" t="n">
         <v>1.6</v>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1056,7 +1192,6 @@
       <c r="I18" t="n">
         <v>1.4</v>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1108,7 +1243,6 @@
       <c r="I20" t="n">
         <v>1.3</v>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1140,7 +1274,6 @@
       <c r="I21" t="n">
         <v>1.2</v>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1172,7 +1305,6 @@
       <c r="I22" t="n">
         <v>1</v>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1204,7 +1336,6 @@
       <c r="I23" t="n">
         <v>1</v>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1236,7 +1367,6 @@
       <c r="I24" t="n">
         <v>0.9</v>
       </c>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1268,7 +1398,6 @@
       <c r="I25" t="n">
         <v>0.8</v>
       </c>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1300,7 +1429,6 @@
       <c r="I26" t="n">
         <v>0.6</v>
       </c>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1332,7 +1460,6 @@
       <c r="I27" t="n">
         <v>0.6</v>
       </c>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1364,7 +1491,6 @@
       <c r="I28" t="n">
         <v>0.6</v>
       </c>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1396,7 +1522,6 @@
       <c r="I29" t="n">
         <v>0.6</v>
       </c>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1428,7 +1553,6 @@
       <c r="I30" t="n">
         <v>0.5</v>
       </c>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1460,7 +1584,6 @@
       <c r="I31" t="n">
         <v>0.5</v>
       </c>
-      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1492,7 +1615,6 @@
       <c r="I32" t="n">
         <v>0.5</v>
       </c>
-      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1524,7 +1646,6 @@
       <c r="I33" t="n">
         <v>0.5</v>
       </c>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1556,7 +1677,6 @@
       <c r="I34" t="n">
         <v>0.5</v>
       </c>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1588,7 +1708,6 @@
       <c r="I35" t="n">
         <v>0.4</v>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1620,7 +1739,6 @@
       <c r="I36" t="n">
         <v>0.4</v>
       </c>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1652,7 +1770,6 @@
       <c r="I37" t="n">
         <v>0.3</v>
       </c>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1684,7 +1801,6 @@
       <c r="I38" t="n">
         <v>0.3</v>
       </c>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1716,7 +1832,6 @@
       <c r="I39" t="n">
         <v>0.3</v>
       </c>
-      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1748,7 +1863,6 @@
       <c r="I40" t="n">
         <v>0.3</v>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1780,7 +1894,6 @@
       <c r="I41" t="n">
         <v>0.3</v>
       </c>
-      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1812,7 +1925,6 @@
       <c r="I42" t="n">
         <v>0.3</v>
       </c>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1844,7 +1956,6 @@
       <c r="I43" t="n">
         <v>0.2</v>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1876,7 +1987,6 @@
       <c r="I44" t="n">
         <v>0.2</v>
       </c>
-      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1932,6 +2042,3536 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G181"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>World military burden, 2025 — military expenditure as a share of GDP (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Country + 'Burden (% of GDP)' feed Excel's Insert → Maps → Filled Map. Cells are shaded to the SIPRI legend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>ISO3</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Burden (% of GDP)</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Legend band</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Afghanistan</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>AFG</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr"/>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>≥ 9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>DZA</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>ARG</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Armenia</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>AUS</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>AUT</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="n"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>No spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>AZE</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Bahamas</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>BHS</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Belarus</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>BLR</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Belize</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>BLZ</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Benin</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>BEN</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>BTN</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr"/>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Bolivia</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>BOL</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>BIH</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Botswana</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>BWA</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>BRA</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Brunei</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>BRN</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Bulgaria</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>BGR</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>BFA</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Burundi</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>BDI</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Cambodia</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>KHM</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>CMR</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Central African Republic</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>CAF</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Chad</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>TCD</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>CHL</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>CHN</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Congo</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>COG</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>CRI</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>No spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>HRV</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Cuba</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>CUB</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr"/>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Cyprus</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>CYP</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>CZE</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>CIV</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Dem. Rep. of the Congo</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>DNK</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D45" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>Djibouti</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>DJI</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D46" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>DOM</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>ECU</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>EGY</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>El Salvador</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>SLV</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>Equatorial Guinea</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>GNQ</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr"/>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Eritrea</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>ERI</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr"/>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D53" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Eswatini</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>SWZ</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D55" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>FJI</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>FIN</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Gabon</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>GAB</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Gambia</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>GMB</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>GEO</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>GHA</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D63" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>GRC</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D64" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Greenland</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>GRL</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr"/>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>GTM</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D66" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>Guinea</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>GIN</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Guinea-Bissau</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>GNB</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>GUY</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D69" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>HTI</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr"/>
+      <c r="D70" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Honduras</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>HND</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>HUN</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Iceland</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>ISL</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="28" t="inlineStr">
+        <is>
+          <t>No spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>IDN</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>IRN</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>IRQ</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>IRL</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D78" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>ISR</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Jamaica</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>JAM</t>
+        </is>
+      </c>
+      <c r="C81" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>JPN</t>
+        </is>
+      </c>
+      <c r="C82" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>JOR</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D83" s="25" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>Kazakhstan</t>
+        </is>
+      </c>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>KAZ</t>
+        </is>
+      </c>
+      <c r="C84" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D84" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>KEN</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+      <c r="B86" s="11" t="inlineStr"/>
+      <c r="C86" s="12" t="inlineStr"/>
+      <c r="D86" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>Kuwait</t>
+        </is>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>KWT</t>
+        </is>
+      </c>
+      <c r="C87" s="12" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D87" s="25" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t>Kyrgyzstan</t>
+        </is>
+      </c>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>KGZ</t>
+        </is>
+      </c>
+      <c r="C88" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D88" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>Laos</t>
+        </is>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>LAO</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr"/>
+      <c r="D89" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
+        <is>
+          <t>Latvia</t>
+        </is>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>LVA</t>
+        </is>
+      </c>
+      <c r="C90" s="12" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D90" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>Lebanon</t>
+        </is>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>LBN</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D91" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>Lesotho</t>
+        </is>
+      </c>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>LSO</t>
+        </is>
+      </c>
+      <c r="C92" s="12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>Liberia</t>
+        </is>
+      </c>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>LBR</t>
+        </is>
+      </c>
+      <c r="C93" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D93" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="inlineStr">
+        <is>
+          <t>Libya</t>
+        </is>
+      </c>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>LBY</t>
+        </is>
+      </c>
+      <c r="C94" s="12" t="inlineStr"/>
+      <c r="D94" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>LTU</t>
+        </is>
+      </c>
+      <c r="C95" s="12" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="B96" s="11" t="inlineStr">
+        <is>
+          <t>LUX</t>
+        </is>
+      </c>
+      <c r="C96" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D96" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="B97" s="11" t="inlineStr">
+        <is>
+          <t>MDG</t>
+        </is>
+      </c>
+      <c r="C97" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D97" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t>Malawi</t>
+        </is>
+      </c>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>MWI</t>
+        </is>
+      </c>
+      <c r="C98" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D98" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>MYS</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>MLI</t>
+        </is>
+      </c>
+      <c r="C100" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D100" s="25" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Mauritania</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>MRT</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>MEX</t>
+        </is>
+      </c>
+      <c r="C102" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D102" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>Moldova</t>
+        </is>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>MDA</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D103" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>Mongolia</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>MNG</t>
+        </is>
+      </c>
+      <c r="C104" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D104" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>Montenegro</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>MNE</t>
+        </is>
+      </c>
+      <c r="C105" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D105" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="C106" s="12" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D106" s="25" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>Mozambique</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>MOZ</t>
+        </is>
+      </c>
+      <c r="C107" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D107" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>MMR</t>
+        </is>
+      </c>
+      <c r="C108" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D108" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>Namibia</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>NAM</t>
+        </is>
+      </c>
+      <c r="C109" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D109" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>NPL</t>
+        </is>
+      </c>
+      <c r="C110" s="12" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>NLD</t>
+        </is>
+      </c>
+      <c r="C111" s="12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>NZL</t>
+        </is>
+      </c>
+      <c r="C112" s="12" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D112" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>Nicaragua</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>NIC</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D113" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>Niger</t>
+        </is>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>NER</t>
+        </is>
+      </c>
+      <c r="C114" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>NGA</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D115" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>North Korea</t>
+        </is>
+      </c>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>PRK</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr"/>
+      <c r="D116" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>North Macedonia</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>MKD</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D117" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>Northern Cyprus</t>
+        </is>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>CYN</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="inlineStr"/>
+      <c r="D118" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>NOR</t>
+        </is>
+      </c>
+      <c r="C119" s="12" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D119" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>Oman</t>
+        </is>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>OMN</t>
+        </is>
+      </c>
+      <c r="C120" s="12" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D120" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C121" s="12" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>Palestine</t>
+        </is>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>PSE</t>
+        </is>
+      </c>
+      <c r="C122" s="12" t="inlineStr"/>
+      <c r="D122" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C123" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" s="28" t="inlineStr">
+        <is>
+          <t>No spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>Papua New Guinea</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="C124" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D124" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>PRY</t>
+        </is>
+      </c>
+      <c r="C125" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C126" s="12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D126" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>PHL</t>
+        </is>
+      </c>
+      <c r="C127" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>POL</t>
+        </is>
+      </c>
+      <c r="C128" s="12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D128" s="25" t="inlineStr">
+        <is>
+          <t>4.0%–5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="C129" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D129" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>QAT</t>
+        </is>
+      </c>
+      <c r="C130" s="12" t="inlineStr"/>
+      <c r="D130" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>ROU</t>
+        </is>
+      </c>
+      <c r="C131" s="12" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D131" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>RUS</t>
+        </is>
+      </c>
+      <c r="C132" s="12" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D132" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>RWA</t>
+        </is>
+      </c>
+      <c r="C133" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D133" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="B134" s="11" t="inlineStr">
+        <is>
+          <t>SAU</t>
+        </is>
+      </c>
+      <c r="C134" s="12" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D134" s="16" t="inlineStr">
+        <is>
+          <t>5.0%–9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>SEN</t>
+        </is>
+      </c>
+      <c r="C135" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D135" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B136" s="11" t="inlineStr">
+        <is>
+          <t>SRB</t>
+        </is>
+      </c>
+      <c r="C136" s="12" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D136" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>SLE</t>
+        </is>
+      </c>
+      <c r="C137" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D137" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>SVK</t>
+        </is>
+      </c>
+      <c r="C138" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="10" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>SVN</t>
+        </is>
+      </c>
+      <c r="C139" s="12" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D139" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
+        <is>
+          <t>Solomon Islands</t>
+        </is>
+      </c>
+      <c r="B140" s="11" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C140" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D140" s="28" t="inlineStr">
+        <is>
+          <t>No spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>Somalia</t>
+        </is>
+      </c>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>SOM</t>
+        </is>
+      </c>
+      <c r="C141" s="12" t="inlineStr"/>
+      <c r="D141" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
+        <is>
+          <t>Somaliland</t>
+        </is>
+      </c>
+      <c r="B142" s="11" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C142" s="12" t="inlineStr"/>
+      <c r="D142" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>ZAF</t>
+        </is>
+      </c>
+      <c r="C143" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D143" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B144" s="11" t="inlineStr">
+        <is>
+          <t>KOR</t>
+        </is>
+      </c>
+      <c r="C144" s="12" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>South Sudan</t>
+        </is>
+      </c>
+      <c r="B145" s="11" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C145" s="12" t="inlineStr"/>
+      <c r="D145" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="B146" s="11" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="C146" s="12" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D146" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="C147" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D147" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="10" t="inlineStr">
+        <is>
+          <t>Sudan</t>
+        </is>
+      </c>
+      <c r="B148" s="11" t="inlineStr">
+        <is>
+          <t>SDN</t>
+        </is>
+      </c>
+      <c r="C148" s="12" t="inlineStr"/>
+      <c r="D148" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>Suriname</t>
+        </is>
+      </c>
+      <c r="B149" s="11" t="inlineStr">
+        <is>
+          <t>SUR</t>
+        </is>
+      </c>
+      <c r="C149" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D149" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="B150" s="11" t="inlineStr">
+        <is>
+          <t>SWE</t>
+        </is>
+      </c>
+      <c r="C150" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D150" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B151" s="11" t="inlineStr">
+        <is>
+          <t>CHE</t>
+        </is>
+      </c>
+      <c r="C151" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D151" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="inlineStr">
+        <is>
+          <t>Syria</t>
+        </is>
+      </c>
+      <c r="B152" s="11" t="inlineStr">
+        <is>
+          <t>SYR</t>
+        </is>
+      </c>
+      <c r="C152" s="12" t="inlineStr"/>
+      <c r="D152" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="B153" s="11" t="inlineStr">
+        <is>
+          <t>TWN</t>
+        </is>
+      </c>
+      <c r="C153" s="12" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D153" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="10" t="inlineStr">
+        <is>
+          <t>Tajikistan</t>
+        </is>
+      </c>
+      <c r="B154" s="11" t="inlineStr">
+        <is>
+          <t>TJK</t>
+        </is>
+      </c>
+      <c r="C154" s="12" t="inlineStr"/>
+      <c r="D154" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
+          <t>TZA</t>
+        </is>
+      </c>
+      <c r="C155" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="10" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="B156" s="11" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="C156" s="12" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D156" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
+        <is>
+          <t>Timor-Leste</t>
+        </is>
+      </c>
+      <c r="B157" s="11" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
+      <c r="C157" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D157" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="10" t="inlineStr">
+        <is>
+          <t>Togo</t>
+        </is>
+      </c>
+      <c r="B158" s="11" t="inlineStr">
+        <is>
+          <t>TGO</t>
+        </is>
+      </c>
+      <c r="C158" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D158" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t>Trinidad and Tobago</t>
+        </is>
+      </c>
+      <c r="B159" s="11" t="inlineStr">
+        <is>
+          <t>TTO</t>
+        </is>
+      </c>
+      <c r="C159" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D159" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="B160" s="11" t="inlineStr">
+        <is>
+          <t>TUN</t>
+        </is>
+      </c>
+      <c r="C160" s="12" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D160" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="B161" s="11" t="inlineStr">
+        <is>
+          <t>TUR</t>
+        </is>
+      </c>
+      <c r="C161" s="12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D161" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="10" t="inlineStr">
+        <is>
+          <t>Turkmenistan</t>
+        </is>
+      </c>
+      <c r="B162" s="11" t="inlineStr">
+        <is>
+          <t>TKM</t>
+        </is>
+      </c>
+      <c r="C162" s="12" t="inlineStr"/>
+      <c r="D162" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="B163" s="11" t="inlineStr">
+        <is>
+          <t>UGA</t>
+        </is>
+      </c>
+      <c r="C163" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D163" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="B164" s="11" t="inlineStr">
+        <is>
+          <t>UKR</t>
+        </is>
+      </c>
+      <c r="C164" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D164" s="8" t="inlineStr">
+        <is>
+          <t>≥ 9.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="B165" s="11" t="inlineStr">
+        <is>
+          <t>ARE</t>
+        </is>
+      </c>
+      <c r="C165" s="12" t="inlineStr"/>
+      <c r="D165" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B166" s="11" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="C166" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D166" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B167" s="11" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C167" s="12" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D167" s="27" t="inlineStr">
+        <is>
+          <t>3.0%–4.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="10" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
+          <t>URY</t>
+        </is>
+      </c>
+      <c r="C168" s="12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D168" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="10" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B169" s="11" t="inlineStr">
+        <is>
+          <t>UZB</t>
+        </is>
+      </c>
+      <c r="C169" s="12" t="inlineStr"/>
+      <c r="D169" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="inlineStr">
+        <is>
+          <t>Vanuatu</t>
+        </is>
+      </c>
+      <c r="B170" s="11" t="inlineStr">
+        <is>
+          <t>VUT</t>
+        </is>
+      </c>
+      <c r="C170" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" s="28" t="inlineStr">
+        <is>
+          <t>No spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="inlineStr">
+        <is>
+          <t>Venezuela</t>
+        </is>
+      </c>
+      <c r="B171" s="11" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="C171" s="12" t="inlineStr"/>
+      <c r="D171" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="10" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="B172" s="11" t="inlineStr">
+        <is>
+          <t>VNM</t>
+        </is>
+      </c>
+      <c r="C172" s="12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D172" s="14" t="inlineStr">
+        <is>
+          <t>2.0%–3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="10" t="inlineStr">
+        <is>
+          <t>Western Sahara</t>
+        </is>
+      </c>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
+          <t>ESH</t>
+        </is>
+      </c>
+      <c r="C173" s="12" t="inlineStr"/>
+      <c r="D173" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="10" t="inlineStr">
+        <is>
+          <t>Yemen</t>
+        </is>
+      </c>
+      <c r="B174" s="11" t="inlineStr">
+        <is>
+          <t>YEM</t>
+        </is>
+      </c>
+      <c r="C174" s="12" t="inlineStr"/>
+      <c r="D174" s="13" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="10" t="inlineStr">
+        <is>
+          <t>Zambia</t>
+        </is>
+      </c>
+      <c r="B175" s="11" t="inlineStr">
+        <is>
+          <t>ZMB</t>
+        </is>
+      </c>
+      <c r="C175" s="12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D175" s="18" t="inlineStr">
+        <is>
+          <t>1.0%–2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="10" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="B176" s="11" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D176" s="20" t="inlineStr">
+        <is>
+          <t>&lt; 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="29" t="inlineStr">
+        <is>
+          <t>'Military burden' is military expenditure as a share of GDP; it represents the relative economic cost of the military.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="29" t="inlineStr">
+        <is>
+          <t>Countries shown as 'No data' are areas where data is unavailable or not reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="29" t="inlineStr">
+        <is>
+          <t>The 40 largest spenders use 2025 GDP-share figures; other countries use the latest available SIPRI figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="29" t="inlineStr">
+        <is>
+          <t>Source: SIPRI Military Expenditure Database, Apr. 2026. Geometry names: Natural Earth.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2059,7 +5699,6 @@
       <c r="F4" t="n">
         <v>1.2</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2084,7 +5723,6 @@
       <c r="F5" t="n">
         <v>0.8</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2134,7 +5772,6 @@
       <c r="F7" t="n">
         <v>0.6</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2159,7 +5796,6 @@
       <c r="F8" t="n">
         <v>34</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2184,7 +5820,6 @@
       <c r="F9" t="n">
         <v>2</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2234,7 +5869,6 @@
       <c r="F11" t="n">
         <v>0.1</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2259,7 +5893,6 @@
       <c r="F12" t="n">
         <v>16</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2284,7 +5917,6 @@
       <c r="F13" t="n">
         <v>1.3</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2309,7 +5941,6 @@
       <c r="F14" t="n">
         <v>3.8</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2334,7 +5965,6 @@
       <c r="F15" t="n">
         <v>2.3</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2384,7 +6014,6 @@
       <c r="F17" t="n">
         <v>20</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2409,7 +6038,6 @@
       <c r="F18" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2445,7 +6073,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2635,7 +6263,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Embed rendered choropleth as 'World Map' sheet in workbook
Add a first-tab 'World Map' sheet with the rendered SIPRI military-burden
map baked in as an image, so the map is visible on open without Excel's
online Filled Map geocoding. embed_map_image.py generates it from the PNG
export of the HTML map.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xaim2Fr7Zv9VVTJ6KQGu17
</commit_message>
<xml_diff>
--- a/SIPRI_Military_Expenditure_2025.xlsx
+++ b/SIPRI_Military_Expenditure_2025.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Top 40 Spenders 2025" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Military Burden Map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Regions &amp; Subregions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="World Share (Top 15)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="World Totals &amp; Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="World Map" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Top 40 Spenders 2025" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Military Burden Map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Regions &amp; Subregions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="World Share (Top 15)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="World Totals &amp; Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -312,6 +313,36 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10001250" cy="6943725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -601,6 +632,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>World military burden, 2025 — military expenditure as a share of GDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Source: SIPRI Military Expenditure Database, Apr. 2026. See the 'Military Burden Map' sheet for the underlying data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2041,7 +2101,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5571,7 +5631,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6073,7 +6133,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6263,7 +6323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>